<commit_message>
Updating example xlsx for IAR-DST v2
</commit_message>
<xml_diff>
--- a/doc/_static/example-files/PMHC-4-0-combined.xlsx
+++ b/doc/_static/example-files/PMHC-4-0-combined.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="695" uniqueCount="347">
   <si>
     <t>key</t>
   </si>
@@ -143,6 +143,9 @@
     <t>BBBBG220219409</t>
   </si>
   <si>
+    <t>C405</t>
+  </si>
+  <si>
     <t>intake_key</t>
   </si>
   <si>
@@ -221,6 +224,9 @@
     <t>I409</t>
   </si>
   <si>
+    <t>I410</t>
+  </si>
+  <si>
     <t>measure_key</t>
   </si>
   <si>
@@ -297,6 +303,15 @@
   </si>
   <si>
     <t>IarDstIM09</t>
+  </si>
+  <si>
+    <t>2.adult</t>
+  </si>
+  <si>
+    <t>IarDstIM10</t>
+  </si>
+  <si>
+    <t>2.child</t>
   </si>
   <si>
     <t>episode_key</t>
@@ -1426,31 +1441,31 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D1" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="E1" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="F1" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="G1" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="H1" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="I1" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="J1" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -1458,10 +1473,10 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="C2" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="D2">
         <v>5</v>
@@ -1487,10 +1502,10 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="C3" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D3">
         <v>2</v>
@@ -1516,10 +1531,10 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="C4" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D4">
         <v>9</v>
@@ -1545,10 +1560,10 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="C5" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1574,10 +1589,10 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="C6" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="D6">
         <v>4</v>
@@ -1603,10 +1618,10 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="C7" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D7">
         <v>4</v>
@@ -1632,10 +1647,10 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="C8" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="D8">
         <v>5</v>
@@ -1661,10 +1676,10 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="C9" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -1690,10 +1705,10 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="C10" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D10">
         <v>3</v>
@@ -1719,10 +1734,10 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="C11" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D11">
         <v>2</v>
@@ -1758,163 +1773,163 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D1" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="E1" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="F1" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="G1" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="H1" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="I1" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="J1" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="K1" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="L1" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="M1" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="N1" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="O1" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="P1" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="Q1" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="R1" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="S1" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="T1" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="U1" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="V1" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="W1" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="X1" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="Y1" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="Z1" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="AA1" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="AB1" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="AC1" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="AD1" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="AE1" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="AF1" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="AG1" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="AH1" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="AI1" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="AJ1" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="AK1" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="AL1" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="AM1" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="AN1" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="AO1" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="AP1" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="AQ1" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="AR1" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="AS1" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="AT1" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="AU1" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="AV1" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="AW1" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="AX1" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="AY1" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="AZ1" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="BA1" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="BB1" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="2" spans="1:54">
@@ -1922,13 +1937,13 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D2" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E2">
         <v>2</v>
@@ -2083,13 +2098,13 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="C3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="D3" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -2244,13 +2259,13 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="C4" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="D4" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2405,13 +2420,13 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="C5" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="D5" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="E5">
         <v>2</v>
@@ -2566,13 +2581,13 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="C6" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="D6" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="E6">
         <v>2</v>
@@ -2727,13 +2742,13 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C7" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="D7" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2888,13 +2903,13 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="C8" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="D8" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -3049,13 +3064,13 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="C9" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="D9" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E9">
         <v>2</v>
@@ -3210,13 +3225,13 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="C10" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="D10" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E10">
         <v>2</v>
@@ -3371,13 +3386,13 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
+        <v>267</v>
+      </c>
+      <c r="C11" t="s">
+        <v>153</v>
+      </c>
+      <c r="D11" t="s">
         <v>262</v>
-      </c>
-      <c r="C11" t="s">
-        <v>148</v>
-      </c>
-      <c r="D11" t="s">
-        <v>257</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -3532,13 +3547,13 @@
         <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="C12" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="D12" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -3693,13 +3708,13 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="C13" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="D13" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -3854,13 +3869,13 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="C14" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D14" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -4015,13 +4030,13 @@
         <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="C15" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D15" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E15">
         <v>2</v>
@@ -4176,13 +4191,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C16" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="D16" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -4337,13 +4352,13 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="C17" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="D17" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="E17">
         <v>2</v>
@@ -4498,13 +4513,13 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="C18" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D18" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="E18">
         <v>2</v>
@@ -4659,13 +4674,13 @@
         <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C19" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="D19" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -4820,13 +4835,13 @@
         <v>15</v>
       </c>
       <c r="B20" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C20" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D20" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="E20">
         <v>1</v>
@@ -4981,13 +4996,13 @@
         <v>15</v>
       </c>
       <c r="B21" t="s">
+        <v>279</v>
+      </c>
+      <c r="C21" t="s">
+        <v>163</v>
+      </c>
+      <c r="D21" t="s">
         <v>274</v>
-      </c>
-      <c r="C21" t="s">
-        <v>158</v>
-      </c>
-      <c r="D21" t="s">
-        <v>269</v>
       </c>
       <c r="E21">
         <v>2</v>
@@ -5142,13 +5157,13 @@
         <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="C22" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="D22" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="E22">
         <v>1</v>
@@ -5313,55 +5328,55 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="C1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="E1" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
       <c r="F1" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="G1" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
       <c r="H1" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="I1" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
       <c r="J1" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="K1" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="L1" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="M1" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="N1" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="O1" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="P1" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="Q1" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="R1" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
     </row>
     <row r="2" spans="1:18">
@@ -5369,10 +5384,10 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="C2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D2">
         <v>17052021</v>
@@ -5411,7 +5426,7 @@
         <v>1</v>
       </c>
       <c r="P2" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="Q2">
         <v>0</v>
@@ -5422,10 +5437,10 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="C3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D3">
         <v>17122021</v>
@@ -5464,7 +5479,7 @@
         <v>1</v>
       </c>
       <c r="P3" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="Q3">
         <v>11</v>
@@ -5475,10 +5490,10 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="C4" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D4">
         <v>28032021</v>
@@ -5517,7 +5532,7 @@
         <v>2</v>
       </c>
       <c r="P4" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="Q4">
         <v>12</v>
@@ -5528,10 +5543,10 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C5" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D5">
         <v>17052021</v>
@@ -5570,7 +5585,7 @@
         <v>2</v>
       </c>
       <c r="P5" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="Q5">
         <v>13</v>
@@ -5581,10 +5596,10 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="C6" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D6">
         <v>3082021</v>
@@ -5623,7 +5638,7 @@
         <v>1</v>
       </c>
       <c r="P6" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="Q6">
         <v>14</v>
@@ -5634,10 +5649,10 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="C7" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D7">
         <v>17112021</v>
@@ -5676,7 +5691,7 @@
         <v>1</v>
       </c>
       <c r="P7" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="Q7">
         <v>0</v>
@@ -5687,10 +5702,10 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="C8" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="D8">
         <v>12082021</v>
@@ -5729,7 +5744,7 @@
         <v>1</v>
       </c>
       <c r="P8" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="Q8">
         <v>11</v>
@@ -5740,10 +5755,10 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="C9" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D9">
         <v>11012022</v>
@@ -5782,7 +5797,7 @@
         <v>2</v>
       </c>
       <c r="P9" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="Q9">
         <v>12</v>
@@ -5793,10 +5808,10 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="C10" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D10">
         <v>28062021</v>
@@ -5835,7 +5850,7 @@
         <v>2</v>
       </c>
       <c r="P10" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="Q10">
         <v>13</v>
@@ -5846,10 +5861,10 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="C11" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D11">
         <v>17082021</v>
@@ -5888,7 +5903,7 @@
         <v>1</v>
       </c>
       <c r="P11" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="Q11">
         <v>0</v>
@@ -5909,16 +5924,16 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="C1" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="D1" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="E1" t="s">
-        <v>312</v>
+        <v>317</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -5926,13 +5941,13 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>313</v>
+        <v>318</v>
       </c>
       <c r="C2" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="D2" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -5943,13 +5958,13 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="C3" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="D3" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -5960,13 +5975,13 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C4" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="D4" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -5977,13 +5992,13 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="C5" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="D5" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="E5">
         <v>1</v>
@@ -5994,13 +6009,13 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="C6" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="D6" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="E6">
         <v>1</v>
@@ -6011,13 +6026,13 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="C7" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
       <c r="D7" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -6028,13 +6043,13 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="C8" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="D8" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -6045,13 +6060,13 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>327</v>
+        <v>332</v>
       </c>
       <c r="C9" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="D9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -6062,13 +6077,13 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="C10" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="D10" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -6079,13 +6094,13 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>331</v>
+        <v>336</v>
       </c>
       <c r="C11" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="D11" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -6096,13 +6111,13 @@
         <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>333</v>
+        <v>338</v>
       </c>
       <c r="C12" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
       <c r="D12" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="E12">
         <v>2</v>
@@ -6113,13 +6128,13 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>334</v>
+        <v>339</v>
       </c>
       <c r="C13" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="D13" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="E13">
         <v>2</v>
@@ -6140,28 +6155,28 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="C1" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="D1" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="E1" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="F1" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="G1" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="H1" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="I1" t="s">
-        <v>341</v>
+        <v>346</v>
       </c>
     </row>
     <row r="2" spans="1:9">
@@ -6169,7 +6184,7 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="C2">
         <v>7</v>
@@ -6195,7 +6210,7 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="C3">
         <v>99</v>
@@ -6221,7 +6236,7 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="C4">
         <v>5</v>
@@ -6247,7 +6262,7 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="C5">
         <v>4</v>
@@ -6273,7 +6288,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="C6">
         <v>4</v>
@@ -6299,7 +6314,7 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="C7">
         <v>9</v>
@@ -6325,7 +6340,7 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>326</v>
+        <v>331</v>
       </c>
       <c r="C8">
         <v>7</v>
@@ -6351,7 +6366,7 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>328</v>
+        <v>333</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -6377,7 +6392,7 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>330</v>
+        <v>335</v>
       </c>
       <c r="C10">
         <v>11</v>
@@ -6403,7 +6418,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>332</v>
+        <v>337</v>
       </c>
       <c r="C11">
         <v>5</v>
@@ -6499,7 +6514,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:11">
@@ -6694,6 +6709,38 @@
         <v>6104</v>
       </c>
       <c r="J6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
+      <c r="A7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7">
+        <v>99999060620162</v>
+      </c>
+      <c r="D7">
+        <v>6062016</v>
+      </c>
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>9</v>
+      </c>
+      <c r="H7">
+        <v>9999</v>
+      </c>
+      <c r="I7">
+        <v>6104</v>
+      </c>
+      <c r="J7">
         <v>1</v>
       </c>
     </row>
@@ -6704,7 +6751,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -6712,43 +6759,43 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C1" t="s">
         <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="I1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="J1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="K1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:14">
@@ -6756,7 +6803,7 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C2" t="s">
         <v>28</v>
@@ -6786,7 +6833,7 @@
         <v>27072021</v>
       </c>
       <c r="L2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="M2" t="s">
         <v>15</v>
@@ -6797,7 +6844,7 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C3" t="s">
         <v>28</v>
@@ -6838,7 +6885,7 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C4" t="s">
         <v>28</v>
@@ -6868,7 +6915,7 @@
         <v>30082021</v>
       </c>
       <c r="L4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M4" t="s">
         <v>15</v>
@@ -6879,7 +6926,7 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C5" t="s">
         <v>28</v>
@@ -6909,7 +6956,7 @@
         <v>3082021</v>
       </c>
       <c r="L5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="M5" t="s">
         <v>15</v>
@@ -6920,7 +6967,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C6" t="s">
         <v>28</v>
@@ -6952,7 +6999,7 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C7" t="s">
         <v>30</v>
@@ -6984,7 +7031,7 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C8" t="s">
         <v>28</v>
@@ -7014,7 +7061,7 @@
         <v>10092021</v>
       </c>
       <c r="L8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="M8" t="s">
         <v>15</v>
@@ -7025,7 +7072,7 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
         <v>32</v>
@@ -7057,7 +7104,7 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C10" t="s">
         <v>34</v>
@@ -7089,7 +7136,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -7114,6 +7161,38 @@
       </c>
       <c r="J11">
         <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>12062024</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>1</v>
+      </c>
+      <c r="I12">
+        <v>12062024</v>
+      </c>
+      <c r="J12">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -7123,7 +7202,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O11"/>
+  <dimension ref="A1:O12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -7131,46 +7210,46 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="F1" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G1" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H1" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="I1" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="J1" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="K1" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="L1" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="M1" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="N1" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="O1" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:15">
@@ -7178,10 +7257,10 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -7211,7 +7290,7 @@
         <v>0</v>
       </c>
       <c r="M2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="N2">
         <v>3</v>
@@ -7222,10 +7301,10 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -7255,7 +7334,7 @@
         <v>0</v>
       </c>
       <c r="M3" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="N3">
         <v>9</v>
@@ -7266,10 +7345,10 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -7310,10 +7389,10 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -7343,7 +7422,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="N5">
         <v>3</v>
@@ -7354,10 +7433,10 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -7398,40 +7477,40 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>2</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>3</v>
+      </c>
+      <c r="L7">
+        <v>2</v>
+      </c>
+      <c r="M7" t="s">
         <v>84</v>
-      </c>
-      <c r="C7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-      <c r="H7">
-        <v>2</v>
-      </c>
-      <c r="I7">
-        <v>2</v>
-      </c>
-      <c r="J7">
-        <v>0</v>
-      </c>
-      <c r="K7">
-        <v>3</v>
-      </c>
-      <c r="L7">
-        <v>2</v>
-      </c>
-      <c r="M7" t="s">
-        <v>82</v>
       </c>
       <c r="N7">
         <v>3</v>
@@ -7442,10 +7521,10 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -7486,10 +7565,10 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D9">
         <v>1</v>
@@ -7530,10 +7609,10 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -7563,7 +7642,7 @@
         <v>4</v>
       </c>
       <c r="M10" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="N10">
         <v>4</v>
@@ -7574,13 +7653,13 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
-      </c>
-      <c r="D11">
-        <v>1</v>
+        <v>64</v>
+      </c>
+      <c r="D11" t="s">
+        <v>92</v>
       </c>
       <c r="E11">
         <v>3</v>
@@ -7607,9 +7686,53 @@
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="N11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15">
+      <c r="A12" t="s">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s">
+        <v>93</v>
+      </c>
+      <c r="C12" t="s">
+        <v>65</v>
+      </c>
+      <c r="D12" t="s">
+        <v>94</v>
+      </c>
+      <c r="E12">
+        <v>3</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>4</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+      <c r="M12" t="s">
+        <v>80</v>
+      </c>
+      <c r="N12">
         <v>3</v>
       </c>
     </row>
@@ -7628,91 +7751,91 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C1" t="s">
         <v>18</v>
       </c>
       <c r="D1" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="E1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F1" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="G1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I1" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="J1" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="K1" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="L1" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="M1" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="N1" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="O1" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="P1" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="Q1" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="R1" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="S1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="T1" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="U1" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="V1" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="W1" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="X1" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="Y1" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="Z1" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="AA1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="AB1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="AC1" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="AD1" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:30">
@@ -7720,7 +7843,7 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C2" t="s">
         <v>28</v>
@@ -7801,7 +7924,7 @@
         <v>7</v>
       </c>
       <c r="AC2" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
     </row>
     <row r="3" spans="1:30">
@@ -7809,7 +7932,7 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C3" t="s">
         <v>28</v>
@@ -7890,10 +8013,10 @@
         <v>4</v>
       </c>
       <c r="AC3" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="AD3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
     </row>
     <row r="4" spans="1:30">
@@ -7901,7 +8024,7 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s">
         <v>30</v>
@@ -7982,7 +8105,7 @@
         <v>4</v>
       </c>
       <c r="AC4" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:30">
@@ -7990,7 +8113,7 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="C5" t="s">
         <v>30</v>
@@ -8071,7 +8194,7 @@
         <v>6</v>
       </c>
       <c r="AC5" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6" spans="1:30">
@@ -8079,7 +8202,7 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C6" t="s">
         <v>32</v>
@@ -8160,7 +8283,7 @@
         <v>8</v>
       </c>
       <c r="AC6" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" spans="1:30">
@@ -8168,7 +8291,7 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C7" t="s">
         <v>32</v>
@@ -8246,7 +8369,7 @@
         <v>8</v>
       </c>
       <c r="AC7" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
     </row>
     <row r="8" spans="1:30">
@@ -8254,7 +8377,7 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C8" t="s">
         <v>34</v>
@@ -8335,7 +8458,7 @@
         <v>5</v>
       </c>
       <c r="AC8" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="1:30">
@@ -8343,7 +8466,7 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="C9" t="s">
         <v>36</v>
@@ -8424,7 +8547,7 @@
         <v>9</v>
       </c>
       <c r="AC9" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:30">
@@ -8432,7 +8555,7 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C10" t="s">
         <v>36</v>
@@ -8513,7 +8636,7 @@
         <v>5</v>
       </c>
       <c r="AC10" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:30">
@@ -8521,7 +8644,7 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C11" t="s">
         <v>36</v>
@@ -8599,7 +8722,7 @@
         <v>8</v>
       </c>
       <c r="AC11" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -8614,16 +8737,16 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C1" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="D1" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:4">
@@ -8631,13 +8754,13 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C2" t="s">
         <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -8645,13 +8768,13 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C3" t="s">
         <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -8659,13 +8782,13 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="C4" t="s">
         <v>15</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -8673,13 +8796,13 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="C5" t="s">
         <v>15</v>
       </c>
       <c r="D5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -8687,13 +8810,13 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="C6" t="s">
         <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -8701,13 +8824,13 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C7" t="s">
         <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -8715,13 +8838,13 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="C8" t="s">
         <v>15</v>
       </c>
       <c r="D8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -8729,13 +8852,13 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="C9" t="s">
         <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -8743,13 +8866,13 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C10" t="s">
         <v>15</v>
       </c>
       <c r="D10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -8757,13 +8880,13 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C11" t="s">
         <v>15</v>
       </c>
       <c r="D11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -8781,19 +8904,19 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="C1" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D1" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="E1" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="F1" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:6">
@@ -8801,10 +8924,10 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="C2" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D2">
         <v>27012021</v>
@@ -8818,10 +8941,10 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C3" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="D3">
         <v>6022021</v>
@@ -8835,10 +8958,10 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="C4" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="D4">
         <v>26092020</v>
@@ -8852,10 +8975,10 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="C5" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D5">
         <v>19012021</v>
@@ -8869,10 +8992,10 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="C6" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D6">
         <v>17032021</v>
@@ -8886,10 +9009,10 @@
         <v>15</v>
       </c>
       <c r="B7" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="C7" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D7">
         <v>20102020</v>
@@ -8903,10 +9026,10 @@
         <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="C8" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D8">
         <v>4062021</v>
@@ -8920,10 +9043,10 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C9" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D9">
         <v>16082020</v>
@@ -8937,10 +9060,10 @@
         <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="C10" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="D10">
         <v>1072021</v>
@@ -8954,10 +9077,10 @@
         <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C11" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="D11">
         <v>26092020</v>
@@ -8971,10 +9094,10 @@
         <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="C12" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="D12">
         <v>6082020</v>
@@ -8988,10 +9111,10 @@
         <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C13" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D13">
         <v>21032021</v>
@@ -9005,10 +9128,10 @@
         <v>15</v>
       </c>
       <c r="B14" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C14" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D14">
         <v>18012021</v>
@@ -9022,10 +9145,10 @@
         <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="C15" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D15">
         <v>21012021</v>
@@ -9039,10 +9162,10 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="C16" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D16">
         <v>17082020</v>
@@ -9056,10 +9179,10 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C17" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="D17">
         <v>15122020</v>
@@ -9073,10 +9196,10 @@
         <v>15</v>
       </c>
       <c r="B18" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C18" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D18">
         <v>22102020</v>
@@ -9090,10 +9213,10 @@
         <v>15</v>
       </c>
       <c r="B19" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="C19" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D19">
         <v>25102020</v>
@@ -9107,10 +9230,10 @@
         <v>15</v>
       </c>
       <c r="B20" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="C20" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D20">
         <v>26042021</v>
@@ -9124,10 +9247,10 @@
         <v>15</v>
       </c>
       <c r="B21" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C21" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="D21">
         <v>19082020</v>
@@ -9141,10 +9264,10 @@
         <v>15</v>
       </c>
       <c r="B22" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C22" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="D22">
         <v>27072021</v>
@@ -9168,58 +9291,58 @@
         <v>5</v>
       </c>
       <c r="B1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C1" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D1" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="E1" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="F1" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="G1" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="H1" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="I1" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="J1" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="K1" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="L1" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="M1" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="N1" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="O1" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="P1" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="Q1" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="R1" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="S1" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:19">
@@ -9227,10 +9350,10 @@
         <v>15</v>
       </c>
       <c r="B2" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C2" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -9283,10 +9406,10 @@
         <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="C3" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="D3">
         <v>3</v>
@@ -9339,10 +9462,10 @@
         <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="C4" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -9395,10 +9518,10 @@
         <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C5" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D5">
         <v>4</v>
@@ -9451,10 +9574,10 @@
         <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C6" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="D6">
         <v>4</v>

</xml_diff>